<commit_message>
feat(sku-search): enhance SKU resolution with exact match query and add quoting function
</commit_message>
<xml_diff>
--- a/features/bulk-update/ImportProducts-Demo.xlsx
+++ b/features/bulk-update/ImportProducts-Demo.xlsx
@@ -1,41 +1,123 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nube\Github\ShopifyOps\features\bulk-update\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE672C4-2EC5-4A1F-965F-9E90F35C145E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+  <si>
+    <t>Command</t>
+  </si>
+  <si>
+    <t>Handle</t>
+  </si>
+  <si>
+    <t>Variant ID</t>
+  </si>
+  <si>
+    <t>Variant SKU</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Variant Price</t>
+  </si>
+  <si>
+    <t>Body HTML</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Vendor</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Tags</t>
+  </si>
+  <si>
+    <t>Tags Command</t>
+  </si>
+  <si>
+    <t>UPDATE</t>
+  </si>
+  <si>
+    <t>snow-globe</t>
+  </si>
+  <si>
+    <t>ACME Gifts</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>6543219870123</t>
+  </si>
+  <si>
+    <t>12.99</t>
+  </si>
+  <si>
+    <t>MERGE</t>
+  </si>
+  <si>
+    <t>24.99</t>
+  </si>
+  <si>
+    <t>gift,seasonal</t>
+  </si>
+  <si>
+    <t>REPLACE</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Updated description.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Snow Globe (test)</t>
+  </si>
+  <si>
+    <t>test-sku</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +147,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,111 +486,113 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Command</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Handle</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Variant ID</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Variant SKU</v>
-      </c>
-      <c r="E1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Variant Price</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Body HTML</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Title</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Vendor</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Tags</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Tags Command</v>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>UPDATE</v>
-      </c>
-      <c r="B2" t="str">
-        <v>snow-globe</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Snow Globe</v>
-      </c>
-      <c r="I2" t="str">
-        <v>ACME Gifts</v>
-      </c>
-      <c r="J2" t="str">
-        <v>active</v>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="3">
-      <c r="C3" t="str">
-        <v>6543219870123</v>
-      </c>
-      <c r="F3" t="str">
-        <v>12.99</v>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>MERGE</v>
-      </c>
-      <c r="D4" t="str">
-        <v>GLOBE-LARGE</v>
-      </c>
-      <c r="F4" t="str">
-        <v>24.99</v>
-      </c>
-      <c r="K4" t="str">
-        <v>gift,seasonal</v>
-      </c>
-      <c r="L4" t="str">
-        <v>REPLACE</v>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>UPDATE</v>
-      </c>
-      <c r="E5" t="str">
-        <v>9876543210</v>
-      </c>
-      <c r="G5" t="str">
-        <v>&lt;p&gt;Updated description.&lt;/p&gt;</v>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>REPLACE</v>
-      </c>
-      <c r="B6" t="str">
-        <v>snow-globe</v>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError sqref="A1:L1 A3:L3 A2 I2:L2 A5:L6 A4:C4 E4:L4 E2:G2 C2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(bulk-update): refactor embedded app to handle bulk updates directly, removing Cloudflare Worker dependency
</commit_message>
<xml_diff>
--- a/features/bulk-update/ImportProducts-Demo.xlsx
+++ b/features/bulk-update/ImportProducts-Demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nube\Github\ShopifyOps\features\bulk-update\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE672C4-2EC5-4A1F-965F-9E90F35C145E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38556E5B-F107-4E5A-813C-67DA02C5A8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>Command</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>test-sku</t>
+  </si>
+  <si>
+    <t>test-product</t>
   </si>
 </sst>
 </file>
@@ -532,6 +535,9 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
       <c r="D2" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
feat(bulk-update): port core business logic + InstalledShopifyClient to app services (#66)
* feat(bulk-update): refactor embedded app to handle bulk updates directly, removing Cloudflare Worker dependency

* feat(bulk-update): port core business logic + InstalledShopifyClient to app services

Ports excel-parser, row-processor, and batch-orchestrator from the
Cloudflare Worker to frontend-shopify-app/app/services/bulk-update/.
Introduces BulkUpdateShopifyClient interface and InstalledShopifyClient
implementation that uses admin.graphql() instead of env-var fetch.

Closes #64

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

---------

Co-authored-by: Ricardo <ilafiukids@gmail.com>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/features/bulk-update/ImportProducts-Demo.xlsx
+++ b/features/bulk-update/ImportProducts-Demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nube\Github\ShopifyOps\features\bulk-update\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE672C4-2EC5-4A1F-965F-9E90F35C145E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38556E5B-F107-4E5A-813C-67DA02C5A8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>Command</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>test-sku</t>
+  </si>
+  <si>
+    <t>test-product</t>
   </si>
 </sst>
 </file>
@@ -532,6 +535,9 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
       <c r="D2" t="s">
         <v>25</v>
       </c>

</xml_diff>